<commit_message>
Update app_main with GPU support, clean config, and latest model checkpoints
</commit_message>
<xml_diff>
--- a/datasets/price_petroleum.xlsx
+++ b/datasets/price_petroleum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03-De tai khoa hoc\Code PetroPrediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F29DC5F-D688-44B3-91CC-C20FECCC662B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED66A7CD-4FF4-473E-8D37-0B496AEF9CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7421B51F-E542-4E2D-BF88-A6A71F6B402C}"/>
   </bookViews>
@@ -249,7 +249,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -270,6 +270,9 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -609,7 +612,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H4643"/>
+  <dimension ref="A1:L4649"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9.4140625" style="1" hidden="1" customWidth="1"/>
@@ -77643,7 +77646,7 @@
         <v>153.61000000000001</v>
       </c>
     </row>
-    <row r="4641" spans="4:8">
+    <row r="4641" spans="4:12">
       <c r="D4641" s="5">
         <v>46135</v>
       </c>
@@ -77660,7 +77663,7 @@
         <v>157.69</v>
       </c>
     </row>
-    <row r="4642" spans="4:8">
+    <row r="4642" spans="4:12">
       <c r="D4642" s="5">
         <v>46136</v>
       </c>
@@ -77677,7 +77680,7 @@
         <v>159.24</v>
       </c>
     </row>
-    <row r="4643" spans="4:8">
+    <row r="4643" spans="4:12">
       <c r="D4643" s="5">
         <v>46139</v>
       </c>
@@ -77692,6 +77695,99 @@
       </c>
       <c r="H4643" s="6">
         <v>160.43</v>
+      </c>
+    </row>
+    <row r="4644" spans="4:12">
+      <c r="D4644" s="5">
+        <v>46140</v>
+      </c>
+      <c r="E4644" s="6">
+        <v>131.54</v>
+      </c>
+      <c r="F4644" s="6">
+        <v>126.52</v>
+      </c>
+      <c r="G4644" s="6">
+        <v>167.39</v>
+      </c>
+      <c r="H4644" s="6">
+        <v>153.79</v>
+      </c>
+      <c r="J4644" s="11"/>
+      <c r="K4644" s="11"/>
+      <c r="L4644" s="11"/>
+    </row>
+    <row r="4645" spans="4:12">
+      <c r="D4645" s="5">
+        <v>46141</v>
+      </c>
+      <c r="E4645" s="6">
+        <v>134.06</v>
+      </c>
+      <c r="F4645" s="6">
+        <v>129.82</v>
+      </c>
+      <c r="G4645" s="6">
+        <v>169.48</v>
+      </c>
+      <c r="H4645" s="6">
+        <v>156.43</v>
+      </c>
+    </row>
+    <row r="4646" spans="4:12">
+      <c r="D4646" s="5">
+        <v>46142</v>
+      </c>
+      <c r="E4646" s="6">
+        <v>137.61000000000001</v>
+      </c>
+      <c r="F4646" s="6">
+        <v>134.27000000000001</v>
+      </c>
+      <c r="G4646" s="6">
+        <v>178.67</v>
+      </c>
+      <c r="H4646" s="6">
+        <v>165.62</v>
+      </c>
+    </row>
+    <row r="4647" spans="4:12">
+      <c r="D4647" s="5">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="4648" spans="4:12">
+      <c r="D4648" s="5">
+        <v>46146</v>
+      </c>
+      <c r="E4648" s="6">
+        <v>133.29</v>
+      </c>
+      <c r="F4648" s="6">
+        <v>130.91999999999999</v>
+      </c>
+      <c r="G4648" s="6">
+        <v>160.72</v>
+      </c>
+      <c r="H4648" s="6">
+        <v>148.76</v>
+      </c>
+    </row>
+    <row r="4649" spans="4:12">
+      <c r="D4649" s="5">
+        <v>46147</v>
+      </c>
+      <c r="E4649" s="6">
+        <v>137.66999999999999</v>
+      </c>
+      <c r="F4649" s="6">
+        <v>136.61000000000001</v>
+      </c>
+      <c r="G4649" s="6">
+        <v>160.59</v>
+      </c>
+      <c r="H4649" s="6">
+        <v>150.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix pyarrow dependency and ensure safe dataframe rendering
</commit_message>
<xml_diff>
--- a/datasets/price_petroleum.xlsx
+++ b/datasets/price_petroleum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03-De tai khoa hoc\Code PetroPrediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED66A7CD-4FF4-473E-8D37-0B496AEF9CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6768489-6953-4154-B44A-FC22D84F0C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7421B51F-E542-4E2D-BF88-A6A71F6B402C}"/>
   </bookViews>
@@ -612,7 +612,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L4649"/>
+  <dimension ref="A1:K4652"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9.4140625" style="1" hidden="1" customWidth="1"/>
@@ -77646,7 +77646,7 @@
         <v>153.61000000000001</v>
       </c>
     </row>
-    <row r="4641" spans="4:12">
+    <row r="4641" spans="4:11">
       <c r="D4641" s="5">
         <v>46135</v>
       </c>
@@ -77663,7 +77663,7 @@
         <v>157.69</v>
       </c>
     </row>
-    <row r="4642" spans="4:12">
+    <row r="4642" spans="4:11">
       <c r="D4642" s="5">
         <v>46136</v>
       </c>
@@ -77680,7 +77680,7 @@
         <v>159.24</v>
       </c>
     </row>
-    <row r="4643" spans="4:12">
+    <row r="4643" spans="4:11">
       <c r="D4643" s="5">
         <v>46139</v>
       </c>
@@ -77697,7 +77697,7 @@
         <v>160.43</v>
       </c>
     </row>
-    <row r="4644" spans="4:12">
+    <row r="4644" spans="4:11">
       <c r="D4644" s="5">
         <v>46140</v>
       </c>
@@ -77713,11 +77713,11 @@
       <c r="H4644" s="6">
         <v>153.79</v>
       </c>
+      <c r="I4644" s="11"/>
       <c r="J4644" s="11"/>
       <c r="K4644" s="11"/>
-      <c r="L4644" s="11"/>
-    </row>
-    <row r="4645" spans="4:12">
+    </row>
+    <row r="4645" spans="4:11">
       <c r="D4645" s="5">
         <v>46141</v>
       </c>
@@ -77734,7 +77734,7 @@
         <v>156.43</v>
       </c>
     </row>
-    <row r="4646" spans="4:12">
+    <row r="4646" spans="4:11">
       <c r="D4646" s="5">
         <v>46142</v>
       </c>
@@ -77751,12 +77751,12 @@
         <v>165.62</v>
       </c>
     </row>
-    <row r="4647" spans="4:12">
+    <row r="4647" spans="4:11">
       <c r="D4647" s="5">
         <v>46143</v>
       </c>
     </row>
-    <row r="4648" spans="4:12">
+    <row r="4648" spans="4:11">
       <c r="D4648" s="5">
         <v>46146</v>
       </c>
@@ -77773,7 +77773,7 @@
         <v>148.76</v>
       </c>
     </row>
-    <row r="4649" spans="4:12">
+    <row r="4649" spans="4:11">
       <c r="D4649" s="5">
         <v>46147</v>
       </c>
@@ -77788,6 +77788,57 @@
       </c>
       <c r="H4649" s="6">
         <v>150.56</v>
+      </c>
+    </row>
+    <row r="4650" spans="4:11">
+      <c r="D4650" s="5">
+        <v>46148</v>
+      </c>
+      <c r="E4650" s="6">
+        <v>134.4</v>
+      </c>
+      <c r="F4650" s="6">
+        <v>133.34</v>
+      </c>
+      <c r="G4650" s="6">
+        <v>157.04</v>
+      </c>
+      <c r="H4650" s="6">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="4651" spans="4:11">
+      <c r="D4651" s="5">
+        <v>46149</v>
+      </c>
+      <c r="E4651" s="6">
+        <v>127.53</v>
+      </c>
+      <c r="F4651" s="6">
+        <v>126.14</v>
+      </c>
+      <c r="G4651" s="6">
+        <v>149.29</v>
+      </c>
+      <c r="H4651" s="6">
+        <v>138.77000000000001</v>
+      </c>
+    </row>
+    <row r="4652" spans="4:11">
+      <c r="D4652" s="5">
+        <v>46150</v>
+      </c>
+      <c r="E4652" s="6">
+        <v>126.06</v>
+      </c>
+      <c r="F4652" s="6">
+        <v>124.48</v>
+      </c>
+      <c r="G4652" s="6">
+        <v>153.97</v>
+      </c>
+      <c r="H4652" s="6">
+        <v>142.94999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: optimize file loading performance, add post-upload manual choice columns, style purple accents, and update batch runner
</commit_message>
<xml_diff>
--- a/datasets/price_petroleum.xlsx
+++ b/datasets/price_petroleum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03-De tai khoa hoc\Code PetroPrediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6768489-6953-4154-B44A-FC22D84F0C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF453E47-D782-42A9-B78A-8FA2BCB8536C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7421B51F-E542-4E2D-BF88-A6A71F6B402C}"/>
   </bookViews>
@@ -612,7 +612,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K4652"/>
+  <dimension ref="A1:K4659"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9.4140625" style="1" hidden="1" customWidth="1"/>
@@ -77841,6 +77841,125 @@
         <v>142.94999999999999</v>
       </c>
     </row>
+    <row r="4653" spans="4:11">
+      <c r="D4653" s="5">
+        <v>46153</v>
+      </c>
+      <c r="E4653" s="6">
+        <v>130.03</v>
+      </c>
+      <c r="F4653" s="6">
+        <v>127.4</v>
+      </c>
+      <c r="G4653" s="6">
+        <v>155.32</v>
+      </c>
+      <c r="H4653" s="6">
+        <v>144.80000000000001</v>
+      </c>
+    </row>
+    <row r="4654" spans="4:11">
+      <c r="D4654" s="5">
+        <v>46154</v>
+      </c>
+      <c r="E4654" s="6">
+        <v>134.72999999999999</v>
+      </c>
+      <c r="F4654" s="6">
+        <v>132.43</v>
+      </c>
+      <c r="G4654" s="6">
+        <v>160.25</v>
+      </c>
+      <c r="H4654" s="6">
+        <v>149.44</v>
+      </c>
+    </row>
+    <row r="4655" spans="4:11">
+      <c r="D4655" s="5">
+        <v>46155</v>
+      </c>
+      <c r="E4655" s="6">
+        <v>137.01</v>
+      </c>
+      <c r="F4655" s="6">
+        <v>134.71</v>
+      </c>
+      <c r="G4655" s="6">
+        <v>165.41</v>
+      </c>
+      <c r="H4655" s="6">
+        <v>154.22999999999999</v>
+      </c>
+    </row>
+    <row r="4656" spans="4:11">
+      <c r="D4656" s="5">
+        <v>46156</v>
+      </c>
+      <c r="E4656" s="6">
+        <v>139.1</v>
+      </c>
+      <c r="F4656" s="6">
+        <v>134.85</v>
+      </c>
+      <c r="G4656" s="6">
+        <v>161.88</v>
+      </c>
+      <c r="H4656" s="6">
+        <v>150.54</v>
+      </c>
+    </row>
+    <row r="4657" spans="4:8">
+      <c r="D4657" s="5">
+        <v>46157</v>
+      </c>
+      <c r="E4657" s="6">
+        <v>139.24</v>
+      </c>
+      <c r="F4657" s="6">
+        <v>135.65</v>
+      </c>
+      <c r="G4657" s="6">
+        <v>163.47</v>
+      </c>
+      <c r="H4657" s="6">
+        <v>152.13</v>
+      </c>
+    </row>
+    <row r="4658" spans="4:8">
+      <c r="D4658" s="5">
+        <v>46160</v>
+      </c>
+      <c r="E4658" s="6">
+        <v>142.12</v>
+      </c>
+      <c r="F4658" s="6">
+        <v>138.63</v>
+      </c>
+      <c r="G4658" s="6">
+        <v>165.04</v>
+      </c>
+      <c r="H4658" s="6">
+        <v>156.26</v>
+      </c>
+    </row>
+    <row r="4659" spans="4:8">
+      <c r="D4659" s="5">
+        <v>46161</v>
+      </c>
+      <c r="E4659" s="6">
+        <v>141.35</v>
+      </c>
+      <c r="F4659" s="6">
+        <v>137.86000000000001</v>
+      </c>
+      <c r="G4659" s="6">
+        <v>166.59</v>
+      </c>
+      <c r="H4659" s="6">
+        <v>159.29</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <autoFilter ref="A1:H3" xr:uid="{6E8F0AB1-E2D8-4E27-8372-67CC5DA2E1D7}">

</xml_diff>